<commit_message>
cambios realizados sobre fuentes y colores, video agregado, mensaje de 60 días agregado
</commit_message>
<xml_diff>
--- a/codigos_invitados.xlsx
+++ b/codigos_invitados.xlsx
@@ -1,26 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x15 xr xr6 xr10">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chewy\OneDrive\Documentos\WEB BODA\web-boda\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User W11\Documents\code\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1D7723A8-081C-4387-B3EA-D70FEF3C0F16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{98C03976-3A25-47E0-B4A5-13016237C4C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="390" yWindow="390" windowWidth="21600" windowHeight="11295"/>
+    <workbookView xWindow="2304" yWindow="2304" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="codigos_invitados" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">codigos_invitados!$A$1:$D$55</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
-  <extLst>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
@@ -132,9 +130,6 @@
     <t>MAY016</t>
   </si>
   <si>
-    <t>Ileana</t>
-  </si>
-  <si>
     <t>MAY017</t>
   </si>
   <si>
@@ -213,9 +208,6 @@
     <t>MAY030</t>
   </si>
   <si>
-    <t>Gabriel/Mayra</t>
-  </si>
-  <si>
     <t>MAY031</t>
   </si>
   <si>
@@ -355,12 +347,18 @@
   </si>
   <si>
     <t>TOTAL</t>
+  </si>
+  <si>
+    <t>Mayra</t>
+  </si>
+  <si>
+    <t>Mariano</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -497,7 +495,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -675,6 +673,12 @@
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.39997558519241921"/>
         <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -838,8 +842,9 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Énfasis1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -899,9 +904,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -939,7 +944,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1045,7 +1050,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1187,18 +1192,21 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D55"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="21.88671875" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1212,11 +1220,11 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="1" t="s">
         <v>5</v>
       </c>
       <c r="C2">
@@ -1226,11 +1234,11 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C3">
@@ -1240,11 +1248,11 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="1" t="s">
         <v>9</v>
       </c>
       <c r="C4">
@@ -1254,11 +1262,11 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="1" t="s">
         <v>11</v>
       </c>
       <c r="C5">
@@ -1268,11 +1276,11 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="1" t="s">
         <v>13</v>
       </c>
       <c r="C6">
@@ -1282,7 +1290,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>14</v>
       </c>
@@ -1296,7 +1304,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>16</v>
       </c>
@@ -1310,7 +1318,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>18</v>
       </c>
@@ -1324,7 +1332,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>20</v>
       </c>
@@ -1338,7 +1346,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>22</v>
       </c>
@@ -1352,25 +1360,25 @@
         <v>4</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A12" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B12" t="s">
-        <v>25</v>
+      <c r="B12" s="1" t="s">
+        <v>108</v>
       </c>
       <c r="C12">
         <v>1</v>
       </c>
       <c r="D12">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A13" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="1" t="s">
         <v>27</v>
       </c>
       <c r="C13">
@@ -1380,11 +1388,11 @@
         <v>6</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A14" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B14" s="1" t="s">
         <v>29</v>
       </c>
       <c r="C14">
@@ -1394,7 +1402,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>30</v>
       </c>
@@ -1408,7 +1416,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>32</v>
       </c>
@@ -1422,12 +1430,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>34</v>
       </c>
       <c r="B17" t="s">
-        <v>35</v>
+        <v>109</v>
       </c>
       <c r="C17">
         <v>1</v>
@@ -1436,12 +1444,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A18" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B18" s="1" t="s">
         <v>36</v>
-      </c>
-      <c r="B18" t="s">
-        <v>37</v>
       </c>
       <c r="C18">
         <v>1</v>
@@ -1450,12 +1458,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A19" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B19" s="1" t="s">
         <v>38</v>
-      </c>
-      <c r="B19" t="s">
-        <v>39</v>
       </c>
       <c r="C19">
         <v>1</v>
@@ -1464,12 +1472,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A20" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B20" s="1" t="s">
         <v>40</v>
-      </c>
-      <c r="B20" t="s">
-        <v>41</v>
       </c>
       <c r="C20">
         <v>1</v>
@@ -1478,12 +1486,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
+        <v>41</v>
+      </c>
+      <c r="B21" t="s">
         <v>42</v>
-      </c>
-      <c r="B21" t="s">
-        <v>43</v>
       </c>
       <c r="C21">
         <v>1</v>
@@ -1492,12 +1500,12 @@
         <v>6</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
+        <v>43</v>
+      </c>
+      <c r="B22" t="s">
         <v>44</v>
-      </c>
-      <c r="B22" t="s">
-        <v>45</v>
       </c>
       <c r="C22">
         <v>3</v>
@@ -1506,12 +1514,12 @@
         <v>8</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
+        <v>45</v>
+      </c>
+      <c r="B23" t="s">
         <v>46</v>
-      </c>
-      <c r="B23" t="s">
-        <v>47</v>
       </c>
       <c r="C23">
         <v>2</v>
@@ -1520,12 +1528,12 @@
         <v>8</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
+        <v>47</v>
+      </c>
+      <c r="B24" t="s">
         <v>48</v>
-      </c>
-      <c r="B24" t="s">
-        <v>49</v>
       </c>
       <c r="C24">
         <v>1</v>
@@ -1534,12 +1542,12 @@
         <v>8</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
+        <v>49</v>
+      </c>
+      <c r="B25" t="s">
         <v>50</v>
-      </c>
-      <c r="B25" t="s">
-        <v>51</v>
       </c>
       <c r="C25">
         <v>2</v>
@@ -1548,12 +1556,12 @@
         <v>8</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
+        <v>51</v>
+      </c>
+      <c r="B26" t="s">
         <v>52</v>
-      </c>
-      <c r="B26" t="s">
-        <v>53</v>
       </c>
       <c r="C26">
         <v>1</v>
@@ -1562,12 +1570,12 @@
         <v>9</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
+        <v>53</v>
+      </c>
+      <c r="B27" t="s">
         <v>54</v>
-      </c>
-      <c r="B27" t="s">
-        <v>55</v>
       </c>
       <c r="C27">
         <v>1</v>
@@ -1576,12 +1584,12 @@
         <v>9</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
+        <v>55</v>
+      </c>
+      <c r="B28" t="s">
         <v>56</v>
-      </c>
-      <c r="B28" t="s">
-        <v>57</v>
       </c>
       <c r="C28">
         <v>1</v>
@@ -1590,12 +1598,12 @@
         <v>9</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
+        <v>57</v>
+      </c>
+      <c r="B29" t="s">
         <v>58</v>
-      </c>
-      <c r="B29" t="s">
-        <v>59</v>
       </c>
       <c r="C29">
         <v>1</v>
@@ -1604,12 +1612,12 @@
         <v>9</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B30" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C30">
         <v>1</v>
@@ -1618,26 +1626,26 @@
         <v>9</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
+        <v>60</v>
+      </c>
+      <c r="B31" t="s">
+        <v>25</v>
+      </c>
+      <c r="C31">
+        <v>1</v>
+      </c>
+      <c r="D31">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
         <v>61</v>
       </c>
-      <c r="B31" t="s">
+      <c r="B32" t="s">
         <v>62</v>
-      </c>
-      <c r="C31">
-        <v>1</v>
-      </c>
-      <c r="D31">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>63</v>
-      </c>
-      <c r="B32" t="s">
-        <v>64</v>
       </c>
       <c r="C32">
         <v>1</v>
@@ -1646,12 +1654,12 @@
         <v>9</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>65</v>
-      </c>
-      <c r="B33" t="s">
-        <v>66</v>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A33" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>64</v>
       </c>
       <c r="C33">
         <v>3</v>
@@ -1660,12 +1668,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>67</v>
-      </c>
-      <c r="B34" t="s">
-        <v>68</v>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A34" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>66</v>
       </c>
       <c r="C34">
         <v>3</v>
@@ -1674,12 +1682,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>69</v>
-      </c>
-      <c r="B35" t="s">
-        <v>70</v>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A35" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>68</v>
       </c>
       <c r="C35">
         <v>3</v>
@@ -1688,12 +1696,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B36" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C36">
         <v>2</v>
@@ -1702,12 +1710,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
-        <v>73</v>
-      </c>
-      <c r="B37" t="s">
-        <v>74</v>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A37" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>72</v>
       </c>
       <c r="C37">
         <v>2</v>
@@ -1716,12 +1724,12 @@
         <v>3</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
-        <v>75</v>
-      </c>
-      <c r="B38" t="s">
-        <v>76</v>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A38" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>74</v>
       </c>
       <c r="C38">
         <v>2</v>
@@ -1730,12 +1738,12 @@
         <v>3</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B39" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C39">
         <v>6</v>
@@ -1744,12 +1752,12 @@
         <v>3</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B40" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C40">
         <v>3</v>
@@ -1758,12 +1766,12 @@
         <v>3</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B41" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C41">
         <v>2</v>
@@ -1772,12 +1780,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B42" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C42">
         <v>3</v>
@@ -1786,12 +1794,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B43" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C43">
         <v>1</v>
@@ -1800,12 +1808,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
-        <v>87</v>
-      </c>
-      <c r="B44" t="s">
-        <v>88</v>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A44" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>86</v>
       </c>
       <c r="C44">
         <v>2</v>
@@ -1814,12 +1822,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B45" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C45">
         <v>1</v>
@@ -1828,12 +1836,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B46" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C46">
         <v>1</v>
@@ -1842,12 +1850,12 @@
         <v>7</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B47" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C47">
         <v>1</v>
@@ -1856,12 +1864,12 @@
         <v>7</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B48" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C48">
         <v>1</v>
@@ -1870,12 +1878,12 @@
         <v>7</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B49" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C49">
         <v>1</v>
@@ -1884,12 +1892,12 @@
         <v>7</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B50" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C50">
         <v>1</v>
@@ -1898,12 +1906,12 @@
         <v>7</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="B51" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C51">
         <v>1</v>
@@ -1912,12 +1920,12 @@
         <v>7</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="B52" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="C52">
         <v>1</v>
@@ -1926,12 +1934,12 @@
         <v>7</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="B53" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C53">
         <v>1</v>
@@ -1940,12 +1948,12 @@
         <v>7</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="B54" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C54">
         <v>1</v>
@@ -1954,15 +1962,16 @@
         <v>3</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C55">
         <v>83</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:D55" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>